<commit_message>
plate3d: the joint example orders one bolt, not two
Grip is 23 at the flange and 22.5 at the web, so length = grip + nut +
proj gave 40.6 and 40.1 - half a millimetre apart, and two lines in the
take-off for a bolt no one buys twice. Both are now written 45, a length
that exists, and proj carries the difference: 7.6 and 8.1 of thread past
the nut. The nut still lands on the steel, because it is measured back
from the shank end.

  M16  F10T  16  45  18  9
</commit_message>
<xml_diff>
--- a/plate3d/PLATE3D_BCJOINT.xlsx
+++ b/plate3d/PLATE3D_BCJOINT.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="95">
   <si>
     <t># PLATE3D  ·  beam-to-column connection, written with SECT</t>
   </si>
@@ -112,22 +112,28 @@
     <t>[nut_h]</t>
   </si>
   <si>
+    <t>[proj]</t>
+  </si>
+  <si>
     <t>#   the point on the MODULE row is the underside of the head, so these start</t>
   </si>
   <si>
     <t>#   on the steel face and the head stands off behind it</t>
   </si>
   <si>
-    <t>#   length = grip + nut + proj. proj is the thread showing past the nut, and</t>
-  </si>
-  <si>
-    <t>#   written longer than that stands its nut off the steel - which is the right</t>
-  </si>
-  <si>
-    <t>#   way for a wrong length to show itself. Grip here is flange + cleat, and</t>
-  </si>
-  <si>
-    <t>#   cleat + web + cleat.</t>
+    <t>#   length = grip + nut + proj, and proj is the thread showing past the nut.</t>
+  </si>
+  <si>
+    <t>#   Grip is flange + cleat, 23, and cleat + web + cleat, 22.5. Bolts come in</t>
+  </si>
+  <si>
+    <t>#   catalogue lengths, so both are written 45 and proj takes up the rest -</t>
+  </si>
+  <si>
+    <t>#   7.6 and 8.1. Left blank proj would be 0.2d and the lengths would come out</t>
+  </si>
+  <si>
+    <t>#   40.6 and 40.1: two take-off lines for a bolt nobody orders twice.</t>
   </si>
   <si>
     <t>BOLT</t>
@@ -677,7 +683,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:P55"/>
+  <dimension ref="B1:P56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -871,7 +877,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>26</v>
       </c>
@@ -902,559 +908,573 @@
       <c r="K12" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="L12" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D19" t="s">
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="E19">
-        <v>16</v>
-      </c>
-      <c r="F19">
-        <v>40.6</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="C20" t="s">
         <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E20">
         <v>16</v>
       </c>
       <c r="F20">
-        <v>40.1</v>
-      </c>
-    </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L20">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="E21">
+        <v>16</v>
+      </c>
+      <c r="F21">
+        <v>45</v>
+      </c>
+      <c r="L21">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F22" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="H23" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="K22" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="L22" s="1" t="s">
+      <c r="J23" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="M22" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="N22" s="1" t="s">
+      <c r="L23" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="O22" s="1" t="s">
+      <c r="M23" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="P22" s="1" t="s">
+      <c r="N23" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23" s="1" t="s">
+      <c r="O23" s="1" t="s">
         <v>57</v>
+      </c>
+      <c r="P23" s="1" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B31" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C31" t="s">
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D31" t="s">
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" t="s">
+        <v>68</v>
+      </c>
+      <c r="D32" t="s">
         <v>19</v>
       </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="G31">
-        <v>0</v>
-      </c>
-      <c r="H31">
-        <v>0</v>
-      </c>
-      <c r="I31" t="s">
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32" t="s">
+        <v>69</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+      <c r="L32">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="J31">
-        <v>0</v>
-      </c>
-      <c r="K31">
-        <v>0</v>
-      </c>
-      <c r="L31">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" t="s">
-        <v>66</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="C33" t="s">
         <v>68</v>
       </c>
-      <c r="E32" t="s">
+      <c r="D33" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33" t="s">
         <v>19</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" t="s">
-        <v>69</v>
-      </c>
-      <c r="D34" t="s">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B35" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" t="s">
+        <v>71</v>
+      </c>
+      <c r="D35" t="s">
         <v>23</v>
       </c>
-      <c r="F34">
-        <v>0</v>
-      </c>
-      <c r="G34">
-        <v>0</v>
-      </c>
-      <c r="H34">
-        <v>0</v>
-      </c>
-      <c r="I34" t="s">
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
+      </c>
+      <c r="I35" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B36" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B35" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" t="s">
-        <v>69</v>
-      </c>
-      <c r="D35" t="s">
-        <v>68</v>
-      </c>
-      <c r="E35" t="s">
+      <c r="E36" t="s">
         <v>23</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F36" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B37" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B40" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B41" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" t="s">
+        <v>42</v>
+      </c>
+      <c r="F41">
+        <v>-45</v>
+      </c>
+      <c r="G41">
+        <v>5</v>
+      </c>
+      <c r="H41">
+        <v>30</v>
+      </c>
+      <c r="I41" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C39" t="s">
-        <v>73</v>
-      </c>
-      <c r="D39" t="s">
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <v>0</v>
+      </c>
+      <c r="N41">
+        <v>0</v>
+      </c>
+      <c r="O41">
+        <v>40</v>
+      </c>
+      <c r="P41">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B42" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" t="s">
+        <v>70</v>
+      </c>
+      <c r="E42" t="s">
         <v>24</v>
       </c>
-      <c r="F39">
-        <v>0</v>
-      </c>
-      <c r="G39">
-        <v>0</v>
-      </c>
-      <c r="H39">
-        <v>0</v>
-      </c>
-      <c r="I39" t="s">
+      <c r="F42" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B44" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B40" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40" t="s">
-        <v>73</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="C44" t="s">
+        <v>76</v>
+      </c>
+      <c r="D44" t="s">
+        <v>44</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44" t="s">
+        <v>77</v>
+      </c>
+      <c r="J44">
+        <v>0</v>
+      </c>
+      <c r="K44">
+        <v>0</v>
+      </c>
+      <c r="L44">
+        <v>0</v>
+      </c>
+      <c r="M44">
+        <v>0</v>
+      </c>
+      <c r="N44">
+        <v>0</v>
+      </c>
+      <c r="O44">
         <v>40</v>
       </c>
-      <c r="F40">
-        <v>-45</v>
-      </c>
-      <c r="G40">
-        <v>5</v>
-      </c>
-      <c r="H40">
-        <v>30</v>
-      </c>
-      <c r="I40" t="s">
+      <c r="P44">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B45" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C45" t="s">
+        <v>76</v>
+      </c>
+      <c r="D45" t="s">
         <v>70</v>
       </c>
-      <c r="J40">
-        <v>0</v>
-      </c>
-      <c r="K40">
-        <v>0</v>
-      </c>
-      <c r="L40">
-        <v>0</v>
-      </c>
-      <c r="M40">
-        <v>0</v>
-      </c>
-      <c r="N40">
-        <v>0</v>
-      </c>
-      <c r="O40">
-        <v>40</v>
-      </c>
-      <c r="P40">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C41" t="s">
-        <v>73</v>
-      </c>
-      <c r="D41" t="s">
-        <v>68</v>
-      </c>
-      <c r="E41" t="s">
-        <v>24</v>
-      </c>
-      <c r="F41" t="s">
+      <c r="E45" t="s">
+        <v>78</v>
+      </c>
+      <c r="F45" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B43" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C43" t="s">
-        <v>74</v>
-      </c>
-      <c r="D43" t="s">
-        <v>42</v>
-      </c>
-      <c r="F43">
-        <v>0</v>
-      </c>
-      <c r="G43">
-        <v>0</v>
-      </c>
-      <c r="H43">
-        <v>0</v>
-      </c>
-      <c r="I43" t="s">
-        <v>75</v>
-      </c>
-      <c r="J43">
-        <v>0</v>
-      </c>
-      <c r="K43">
-        <v>0</v>
-      </c>
-      <c r="L43">
-        <v>0</v>
-      </c>
-      <c r="M43">
-        <v>0</v>
-      </c>
-      <c r="N43">
-        <v>0</v>
-      </c>
-      <c r="O43">
-        <v>40</v>
-      </c>
-      <c r="P43">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B44" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C44" t="s">
-        <v>74</v>
-      </c>
-      <c r="D44" t="s">
-        <v>68</v>
-      </c>
-      <c r="E44" t="s">
-        <v>76</v>
-      </c>
-      <c r="F44" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B46" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C46" s="1" t="s">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F46" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G46" s="1" t="s">
+      <c r="E47" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="H46" s="1" t="s">
+      <c r="F47" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="I46" s="1" t="s">
+      <c r="G47" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B47" s="2" t="s">
+      <c r="H47" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C47" t="s">
+      <c r="I47" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="D47" t="s">
-        <v>66</v>
-      </c>
-      <c r="E47" t="s">
-        <v>86</v>
-      </c>
-      <c r="F47">
-        <v>0</v>
-      </c>
-      <c r="G47">
-        <v>0</v>
-      </c>
-      <c r="H47">
-        <v>-800</v>
       </c>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C48" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D48" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E48" t="s">
+        <v>88</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
+        <v>-800</v>
+      </c>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B49" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F48">
+      <c r="C49" t="s">
+        <v>87</v>
+      </c>
+      <c r="D49" t="s">
+        <v>71</v>
+      </c>
+      <c r="E49" t="s">
+        <v>88</v>
+      </c>
+      <c r="F49">
         <v>160</v>
       </c>
-      <c r="G48">
-        <v>0</v>
-      </c>
-      <c r="H48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B49" s="1" t="s">
-        <v>87</v>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B51" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B52" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C52" t="s">
+        <v>91</v>
+      </c>
+      <c r="D52" t="s">
+        <v>75</v>
+      </c>
+      <c r="E52" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B51" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C51" t="s">
-        <v>89</v>
-      </c>
-      <c r="D51" t="s">
-        <v>73</v>
-      </c>
-      <c r="E51" t="s">
+      <c r="F52">
+        <v>180</v>
+      </c>
+      <c r="G52">
+        <v>33.25</v>
+      </c>
+      <c r="H52">
+        <v>-70</v>
+      </c>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B53" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F51">
-        <v>180</v>
-      </c>
-      <c r="G51">
-        <v>33.25</v>
-      </c>
-      <c r="H51">
-        <v>-70</v>
-      </c>
-    </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B52" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C52" t="s">
-        <v>90</v>
-      </c>
-      <c r="D52" t="s">
-        <v>89</v>
-      </c>
-      <c r="E52" t="s">
+      <c r="C53" t="s">
+        <v>92</v>
+      </c>
+      <c r="D53" t="s">
         <v>91</v>
       </c>
-      <c r="F52">
-        <v>0</v>
-      </c>
-      <c r="G52">
-        <v>0</v>
-      </c>
-      <c r="H52">
-        <v>0</v>
-      </c>
-      <c r="I52" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B53" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C53" t="s">
-        <v>85</v>
-      </c>
-      <c r="D53" t="s">
-        <v>74</v>
-      </c>
       <c r="E53" t="s">
+        <v>93</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B54" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F53">
+      <c r="C54" t="s">
+        <v>87</v>
+      </c>
+      <c r="D54" t="s">
+        <v>76</v>
+      </c>
+      <c r="E54" t="s">
+        <v>88</v>
+      </c>
+      <c r="F54">
         <v>185</v>
       </c>
-      <c r="G53">
+      <c r="G54">
         <v>11.25</v>
       </c>
-      <c r="H53">
+      <c r="H54">
         <v>-40</v>
       </c>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B55" s="2" t="s">
-        <v>92</v>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>